<commit_message>
Ajustes finais do código-fonte para langchaing e LLM gratuito
</commit_message>
<xml_diff>
--- a/templates/matriz_planejamento_template.xlsx
+++ b/templates/matriz_planejamento_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Fabiana\Mestrado IDP\IA Generativa\TrabalhoFinal\AuditGen\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0EC4994-F4BD-46FB-9D2F-145565C77F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B33BC01-A8CC-4764-A342-BFDCD78991C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{408AE258-C170-4A74-B862-F238E137C4ED}"/>
   </bookViews>
@@ -152,6 +152,9 @@
     <t>UNIDADES AUDITADAS: {{unidades_auditadas}}</t>
   </si>
   <si>
+    <t>{{equipe}}</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">REVISADO POR: </t>
     </r>
@@ -164,11 +167,8 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Larissa Maria Ferreira Morais Napoleão Nogueira (matrícula 319357) ou Adileide Ferreira Ribeiro (matrícula 309877)</t>
+      <t>Chefia (matrícula)</t>
     </r>
-  </si>
-  <si>
-    <t>{{equipe}}</t>
   </si>
 </sst>
 </file>
@@ -908,7 +908,7 @@
     </row>
     <row r="4" spans="1:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="33"/>
       <c r="C4" s="33"/>
@@ -1015,7 +1015,7 @@
       <c r="G9" s="5"/>
       <c r="H9" s="13"/>
       <c r="I9" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J9" s="5"/>
       <c r="K9" s="13"/>
@@ -1030,7 +1030,7 @@
       <c r="G10" s="5"/>
       <c r="H10" s="13"/>
       <c r="I10" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J10" s="5"/>
       <c r="K10" s="13"/>
@@ -1045,7 +1045,7 @@
       <c r="G11" s="5"/>
       <c r="H11" s="13"/>
       <c r="I11" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J11" s="5"/>
       <c r="K11" s="13"/>
@@ -1060,7 +1060,7 @@
       <c r="G12" s="5"/>
       <c r="H12" s="13"/>
       <c r="I12" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J12" s="5"/>
       <c r="K12" s="13"/>
@@ -1075,7 +1075,7 @@
       <c r="G13" s="5"/>
       <c r="H13" s="13"/>
       <c r="I13" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J13" s="5"/>
       <c r="K13" s="13"/>
@@ -1090,7 +1090,7 @@
       <c r="G14" s="5"/>
       <c r="H14" s="13"/>
       <c r="I14" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J14" s="5"/>
       <c r="K14" s="18"/>
@@ -1105,7 +1105,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="13"/>
       <c r="I15" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J15" s="5"/>
       <c r="K15" s="18"/>
@@ -1120,7 +1120,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="13"/>
       <c r="I16" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J16" s="5"/>
       <c r="K16" s="18"/>
@@ -1135,7 +1135,7 @@
       <c r="G17" s="10"/>
       <c r="H17" s="13"/>
       <c r="I17" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J17" s="5"/>
       <c r="K17" s="18"/>
@@ -1150,7 +1150,7 @@
       <c r="G18" s="10"/>
       <c r="H18" s="18"/>
       <c r="I18" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J18" s="5"/>
       <c r="K18" s="18"/>
@@ -1165,7 +1165,7 @@
       <c r="G19" s="10"/>
       <c r="H19" s="18"/>
       <c r="I19" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J19" s="5"/>
       <c r="K19" s="18"/>
@@ -1180,7 +1180,7 @@
       <c r="G20" s="12"/>
       <c r="H20" s="19"/>
       <c r="I20" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J20" s="5"/>
       <c r="K20" s="19"/>
@@ -1195,7 +1195,7 @@
       <c r="G21" s="12"/>
       <c r="H21" s="19"/>
       <c r="I21" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J21" s="5"/>
       <c r="K21" s="19"/>
@@ -1210,7 +1210,7 @@
       <c r="G22" s="12"/>
       <c r="H22" s="19"/>
       <c r="I22" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J22" s="5"/>
       <c r="K22" s="19"/>
@@ -1225,7 +1225,7 @@
       <c r="G23" s="12"/>
       <c r="H23" s="19"/>
       <c r="I23" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J23" s="5"/>
       <c r="K23" s="19"/>
@@ -1240,7 +1240,7 @@
       <c r="G24" s="12"/>
       <c r="H24" s="19"/>
       <c r="I24" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J24" s="5"/>
       <c r="K24" s="19"/>
@@ -1255,7 +1255,7 @@
       <c r="G25" s="12"/>
       <c r="H25" s="19"/>
       <c r="I25" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J25" s="5"/>
       <c r="K25" s="19"/>
@@ -1270,7 +1270,7 @@
       <c r="G26" s="12"/>
       <c r="H26" s="19"/>
       <c r="I26" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J26" s="5"/>
       <c r="K26" s="19"/>
@@ -1285,7 +1285,7 @@
       <c r="G27" s="12"/>
       <c r="H27" s="19"/>
       <c r="I27" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J27" s="5"/>
       <c r="K27" s="19"/>
@@ -1300,7 +1300,7 @@
       <c r="G28" s="12"/>
       <c r="H28" s="19"/>
       <c r="I28" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J28" s="5"/>
       <c r="K28" s="19"/>
@@ -1315,7 +1315,7 @@
       <c r="G29" s="12"/>
       <c r="H29" s="19"/>
       <c r="I29" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J29" s="5"/>
       <c r="K29" s="19"/>
@@ -1330,7 +1330,7 @@
       <c r="G30" s="12"/>
       <c r="H30" s="19"/>
       <c r="I30" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J30" s="5"/>
       <c r="K30" s="19"/>
@@ -1345,7 +1345,7 @@
       <c r="G31" s="12"/>
       <c r="H31" s="19"/>
       <c r="I31" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J31" s="5"/>
       <c r="K31" s="19"/>
@@ -1360,7 +1360,7 @@
       <c r="G32" s="12"/>
       <c r="H32" s="19"/>
       <c r="I32" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J32" s="5"/>
       <c r="K32" s="19"/>
@@ -1375,7 +1375,7 @@
       <c r="G33" s="12"/>
       <c r="H33" s="19"/>
       <c r="I33" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="19"/>
@@ -1390,7 +1390,7 @@
       <c r="G34" s="12"/>
       <c r="H34" s="19"/>
       <c r="I34" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J34" s="5"/>
       <c r="K34" s="19"/>
@@ -1405,7 +1405,7 @@
       <c r="G35" s="12"/>
       <c r="H35" s="19"/>
       <c r="I35" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J35" s="5"/>
       <c r="K35" s="19"/>
@@ -1420,7 +1420,7 @@
       <c r="G36" s="12"/>
       <c r="H36" s="19"/>
       <c r="I36" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J36" s="5"/>
       <c r="K36" s="19"/>
@@ -1435,7 +1435,7 @@
       <c r="G37" s="12"/>
       <c r="H37" s="19"/>
       <c r="I37" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J37" s="5"/>
       <c r="K37" s="19"/>
@@ -1450,7 +1450,7 @@
       <c r="G38" s="12"/>
       <c r="H38" s="19"/>
       <c r="I38" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J38" s="5"/>
       <c r="K38" s="19"/>
@@ -1465,7 +1465,7 @@
       <c r="G39" s="12"/>
       <c r="H39" s="19"/>
       <c r="I39" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J39" s="5"/>
       <c r="K39" s="19"/>
@@ -1480,7 +1480,7 @@
       <c r="G40" s="12"/>
       <c r="H40" s="19"/>
       <c r="I40" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J40" s="5"/>
       <c r="K40" s="19"/>
@@ -1495,7 +1495,7 @@
       <c r="G41" s="12"/>
       <c r="H41" s="19"/>
       <c r="I41" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J41" s="5"/>
       <c r="K41" s="19"/>
@@ -1510,7 +1510,7 @@
       <c r="G42" s="12"/>
       <c r="H42" s="19"/>
       <c r="I42" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J42" s="5"/>
       <c r="K42" s="19"/>
@@ -1525,7 +1525,7 @@
       <c r="G43" s="12"/>
       <c r="H43" s="19"/>
       <c r="I43" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J43" s="5"/>
       <c r="K43" s="19"/>
@@ -1540,7 +1540,7 @@
       <c r="G44" s="12"/>
       <c r="H44" s="19"/>
       <c r="I44" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J44" s="5"/>
       <c r="K44" s="19"/>
@@ -1555,7 +1555,7 @@
       <c r="G45" s="12"/>
       <c r="H45" s="19"/>
       <c r="I45" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J45" s="5"/>
       <c r="K45" s="19"/>
@@ -1570,7 +1570,7 @@
       <c r="G46" s="12"/>
       <c r="H46" s="19"/>
       <c r="I46" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J46" s="5"/>
       <c r="K46" s="19"/>
@@ -1585,7 +1585,7 @@
       <c r="G47" s="12"/>
       <c r="H47" s="19"/>
       <c r="I47" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J47" s="5"/>
       <c r="K47" s="19"/>
@@ -1600,7 +1600,7 @@
       <c r="G48" s="12"/>
       <c r="H48" s="19"/>
       <c r="I48" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J48" s="5"/>
       <c r="K48" s="19"/>
@@ -1615,7 +1615,7 @@
       <c r="G49" s="12"/>
       <c r="H49" s="19"/>
       <c r="I49" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J49" s="5"/>
       <c r="K49" s="19"/>
@@ -1630,7 +1630,7 @@
       <c r="G50" s="22"/>
       <c r="H50" s="24"/>
       <c r="I50" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J50" s="22"/>
       <c r="K50" s="24"/>
@@ -1645,7 +1645,7 @@
       <c r="G51" s="22"/>
       <c r="H51" s="24"/>
       <c r="I51" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J51" s="22"/>
       <c r="K51" s="24"/>
@@ -1660,7 +1660,7 @@
       <c r="G52" s="22"/>
       <c r="H52" s="24"/>
       <c r="I52" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J52" s="22"/>
       <c r="K52" s="24"/>
@@ -1675,7 +1675,7 @@
       <c r="G53" s="22"/>
       <c r="H53" s="24"/>
       <c r="I53" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J53" s="22"/>
       <c r="K53" s="24"/>
@@ -1690,7 +1690,7 @@
       <c r="G54" s="22"/>
       <c r="H54" s="24"/>
       <c r="I54" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J54" s="22"/>
       <c r="K54" s="24"/>
@@ -1713,6 +1713,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="f8e977c5-1382-4d06-a69c-9787a52d7675" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C1BE48FA3000F34A913629A2C4BE2A6B" ma:contentTypeVersion="15" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="1b415bcf9c0f9c00a3de6003c90a4927">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7" xmlns:ns3="f8e977c5-1382-4d06-a69c-9787a52d7675" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a0ac9549459b4879b8f45b25f824cf63" ns2:_="" ns3:_="">
     <xsd:import namespace="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7"/>
@@ -1947,41 +1967,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="f8e977c5-1382-4d06-a69c-9787a52d7675" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D57EDFE-63A6-4119-B9C0-8C86EEDE4CAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C739CA6C-854F-4521-9D38-76E2CDDABE58}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7"/>
-    <ds:schemaRef ds:uri="f8e977c5-1382-4d06-a69c-9787a52d7675"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2004,9 +1993,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C739CA6C-854F-4521-9D38-76E2CDDABE58}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D57EDFE-63A6-4119-B9C0-8C86EEDE4CAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="cafa2f08-7da3-4c0e-9ece-55bccef3ffa7"/>
+    <ds:schemaRef ds:uri="f8e977c5-1382-4d06-a69c-9787a52d7675"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>